<commit_message>
impl phase 1 desktop app
</commit_message>
<xml_diff>
--- a/wiki/desktop/desktop-development-plan.xlsx
+++ b/wiki/desktop/desktop-development-plan.xlsx
@@ -691,7 +691,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Offline-first Electron desktop client. Local SQLite is the source of truth; Notion is a bidirectional mirror. Phase 0 complete and verified on 2026-07-21 (scaffold + HMR, local SQLite + migrations, domain derivations, IPC skeleton).</t>
+          <t>Offline-first Electron desktop client. Local SQLite is the source of truth; Notion is a bidirectional mirror. Phases 0-1 complete and verified on 2026-07-21: the app is a fully usable offline daily driver (local CRUD, real-time derived balances, 9 sections, multi-window). Next: Phase 2 (Notion onboarding + push).</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       </c>
       <c r="D5" s="5">
         <f>COUNTIF('Development Plan'!$E$5:$E$100,"Done")</f>
-        <v>4</v>
+        <v>9</v>
         <v/>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="F5" s="6">
         <f>IFERROR(D5/B5,0)</f>
-        <v>0.181818181818</v>
+        <v>0.409090909091</v>
         <v/>
       </c>
     </row>
@@ -818,7 +818,7 @@
       </c>
       <c r="C10" s="9">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 1",'Development Plan'!$E$5:$E$100,"Not Started")</f>
-        <v>5</v>
+        <v>0</v>
         <v/>
       </c>
       <c r="D10" s="9">
@@ -828,7 +828,7 @@
       </c>
       <c r="E10" s="9">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 1",'Development Plan'!$E$5:$E$100,"Done")</f>
-        <v>0</v>
+        <v>5</v>
         <v/>
       </c>
       <c r="F10" s="9">
@@ -978,7 +978,7 @@
       </c>
       <c r="C15" s="11">
         <f>SUM(C9:C14)</f>
-        <v>18</v>
+        <v>13</v>
         <v/>
       </c>
       <c r="D15" s="11">
@@ -988,7 +988,7 @@
       </c>
       <c r="E15" s="11">
         <f>SUM(E9:E14)</f>
-        <v>4</v>
+        <v>9</v>
         <v/>
       </c>
       <c r="F15" s="11">
@@ -1054,12 +1054,12 @@
       </c>
       <c r="D19" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 0",'Development Plan'!$E$5:$E$100,"Done")+COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 1",'Development Plan'!$E$5:$E$100,"Done")</f>
-        <v>4</v>
+        <v>9</v>
         <v/>
       </c>
       <c r="E19" s="15">
         <f>IFERROR(D19/C19,0)</f>
-        <v>0.444444444444</v>
+        <v>1.0</v>
         <v/>
       </c>
       <c r="F19" s="16" t="inlineStr">
@@ -1466,10 +1466,14 @@
       </c>
       <c r="E9" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F9" s="24" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F9" s="24" t="inlineStr">
+        <is>
+          <t>Verified 2026-07-21: schema completed with pasabuy columns (migration 0001); all tables + sync columns per local-data-schema.md.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="23" t="inlineStr">
@@ -1494,10 +1498,14 @@
       </c>
       <c r="E10" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F10" s="24" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F10" s="24" t="inlineStr">
+        <is>
+          <t>Verified 2026-07-21: repositories with instant writes, sync_state=dirty, mutation_queue journal, soft-delete via title rewrite; validation in main; full IPC surface. Live-run harness exercised create/update/soft-delete.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="23" t="inlineStr">
@@ -1522,10 +1530,14 @@
       </c>
       <c r="E11" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F11" s="24" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F11" s="24" t="inlineStr">
+        <is>
+          <t>Verified 2026-07-21: live golden checks PASS (income 50,000 / expense 11,500 / margin 38,500 / cash flow 73,000; credit balance -8,000, available 42,000); recompute + derived:updated on every edit; 27 unit tests green.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="23" t="inlineStr">
@@ -1550,10 +1562,14 @@
       </c>
       <c r="E12" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F12" s="24" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F12" s="24" t="inlineStr">
+        <is>
+          <t>Verified 2026-07-21: all 9 sections render from local SQLite over window.api with the web view semantics (fixed categories Transfer/CC Payment/Savings, receivables = no account, income excludes auxiliary). Re-expressed UI (not pixel-ported); full CRUD forms + scheduler panel.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="23" t="inlineStr">
@@ -1578,10 +1594,14 @@
       </c>
       <c r="E13" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F13" s="24" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F13" s="24" t="inlineStr">
+        <is>
+          <t>Verified 2026-07-21: New Window (menu Cmd/Ctrl+N + IPC); records:changed/derived:updated broadcast to all windows; live run showed 2 windows each receiving all 18 events and refetching.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="23" t="inlineStr">

</xml_diff>

<commit_message>
feat: impl phase 2 desktop app
</commit_message>
<xml_diff>
--- a/wiki/desktop/desktop-development-plan.xlsx
+++ b/wiki/desktop/desktop-development-plan.xlsx
@@ -691,7 +691,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Offline-first Electron desktop client. Local SQLite is the source of truth; Notion is a bidirectional mirror. Phases 0-1 complete and verified on 2026-07-21: the app is a fully usable offline daily driver (local CRUD, real-time derived balances, 9 sections, multi-window). Next: Phase 2 (Notion onboarding + push).</t>
+          <t>Offline-first Electron desktop client. Local SQLite is the source of truth; Notion is a bidirectional mirror. Phases 0-2 complete on 2026-07-21: usable offline app + Notion connect (keychain token), schema verification, and idempotent push with rate-limit backoff (verified against a mock Notion API). Next: Phase 3 (pull).</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       </c>
       <c r="D5" s="5">
         <f>COUNTIF('Development Plan'!$E$5:$E$100,"Done")</f>
-        <v>9</v>
+        <v>12</v>
         <v/>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="F5" s="6">
         <f>IFERROR(D5/B5,0)</f>
-        <v>0.409090909091</v>
+        <v>0.545454545455</v>
         <v/>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="C11" s="9">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 2",'Development Plan'!$E$5:$E$100,"Not Started")</f>
-        <v>3</v>
+        <v>0</v>
         <v/>
       </c>
       <c r="D11" s="9">
@@ -860,7 +860,7 @@
       </c>
       <c r="E11" s="9">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 2",'Development Plan'!$E$5:$E$100,"Done")</f>
-        <v>0</v>
+        <v>3</v>
         <v/>
       </c>
       <c r="F11" s="9">
@@ -978,7 +978,7 @@
       </c>
       <c r="C15" s="11">
         <f>SUM(C9:C14)</f>
-        <v>13</v>
+        <v>10</v>
         <v/>
       </c>
       <c r="D15" s="11">
@@ -988,7 +988,7 @@
       </c>
       <c r="E15" s="11">
         <f>SUM(E9:E14)</f>
-        <v>9</v>
+        <v>12</v>
         <v/>
       </c>
       <c r="F15" s="11">
@@ -1086,12 +1086,12 @@
       </c>
       <c r="D20" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 2",'Development Plan'!$E$5:$E$100,"Done")+COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 3",'Development Plan'!$E$5:$E$100,"Done")</f>
-        <v>0</v>
+        <v>3</v>
         <v/>
       </c>
       <c r="E20" s="15">
         <f>IFERROR(D20/C20,0)</f>
-        <v>0.0</v>
+        <v>0.5</v>
         <v/>
       </c>
       <c r="F20" s="16" t="inlineStr">
@@ -1626,10 +1626,14 @@
       </c>
       <c r="E14" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F14" s="24" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F14" s="24" t="inlineStr">
+        <is>
+          <t>Verified 2026-07-21: token validated then encrypted via safeStorage (OS keychain) in userData; no IPC getter returns it. Discovery + per-resource mapping persisted in app_settings. End-to-end against a mock Notion API.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="23" t="inlineStr">
@@ -1654,10 +1658,14 @@
       </c>
       <c r="E15" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F15" s="24" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F15" s="24" t="inlineStr">
+        <is>
+          <t>Verified 2026-07-21: per-resource drift report from the canonical field taxonomy — writable drift = error, computed drift = warning; verify passed on the mock workspace; drift cases covered by unit tests. Real-workspace verify pending the user's token.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="23" t="inlineStr">
@@ -1682,10 +1690,14 @@
       </c>
       <c r="E16" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F16" s="24" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F16" s="24" t="inlineStr">
+        <is>
+          <t>Verified 2026-07-21 against mock Notion API: 3 dirty records created (one absorbed an injected 429 via backoff), page ids + base_snapshot stored, sync_state=clean; edit pushed exactly 1 update (idempotent); empty pass = 0 requests. Local→Notion relation translation with skip-until-linked. Real-workspace push pending the user's token.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="23" t="inlineStr">

</xml_diff>

<commit_message>
feat: impl phase 3 dektop app
</commit_message>
<xml_diff>
--- a/wiki/desktop/desktop-development-plan.xlsx
+++ b/wiki/desktop/desktop-development-plan.xlsx
@@ -691,7 +691,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Offline-first Electron desktop client. Local SQLite is the source of truth; Notion is a bidirectional mirror. Phases 0-2 complete on 2026-07-21: usable offline app + Notion connect (keychain token), schema verification, and idempotent push with rate-limit backoff (verified against a mock Notion API). Next: Phase 3 (pull).</t>
+          <t>Offline-first Electron desktop client. Local SQLite is the source of truth; Notion is a bidirectional mirror. Phases 0-3 complete on 2026-07-21: usable offline app + full Notion sync — connect (keychain token), schema verify, push, and initial + incremental pull (verified vs a mock Notion API). Milestone M2 (backup sync) done. Next: Phase 4 (three-way merge + conflict resolver).</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       </c>
       <c r="D5" s="5">
         <f>COUNTIF('Development Plan'!$E$5:$E$100,"Done")</f>
-        <v>12</v>
+        <v>15</v>
         <v/>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="F5" s="6">
         <f>IFERROR(D5/B5,0)</f>
-        <v>0.545454545455</v>
+        <v>0.681818181818</v>
         <v/>
       </c>
     </row>
@@ -882,7 +882,7 @@
       </c>
       <c r="C12" s="9">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 3",'Development Plan'!$E$5:$E$100,"Not Started")</f>
-        <v>3</v>
+        <v>0</v>
         <v/>
       </c>
       <c r="D12" s="9">
@@ -892,7 +892,7 @@
       </c>
       <c r="E12" s="9">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 3",'Development Plan'!$E$5:$E$100,"Done")</f>
-        <v>0</v>
+        <v>3</v>
         <v/>
       </c>
       <c r="F12" s="9">
@@ -978,7 +978,7 @@
       </c>
       <c r="C15" s="11">
         <f>SUM(C9:C14)</f>
-        <v>10</v>
+        <v>7</v>
         <v/>
       </c>
       <c r="D15" s="11">
@@ -988,7 +988,7 @@
       </c>
       <c r="E15" s="11">
         <f>SUM(E9:E14)</f>
-        <v>12</v>
+        <v>15</v>
         <v/>
       </c>
       <c r="F15" s="11">
@@ -1086,12 +1086,12 @@
       </c>
       <c r="D20" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 2",'Development Plan'!$E$5:$E$100,"Done")+COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 3",'Development Plan'!$E$5:$E$100,"Done")</f>
-        <v>3</v>
+        <v>6</v>
         <v/>
       </c>
       <c r="E20" s="15">
         <f>IFERROR(D20/C20,0)</f>
-        <v>0.5</v>
+        <v>1.0</v>
         <v/>
       </c>
       <c r="F20" s="16" t="inlineStr">
@@ -1722,10 +1722,14 @@
       </c>
       <c r="E17" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F17" s="24" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F17" s="24" t="inlineStr">
+        <is>
+          <t>Verified 2026-07-21 vs mock: full pull inserted 5 reference rows + 2 records into an empty store; Notion relation ids translated to local ids; derived balances correct from pulled records (BPI 70,000).</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="23" t="inlineStr">
@@ -1740,7 +1744,7 @@
       </c>
       <c r="C18" s="24" t="inlineStr">
         <is>
-          <t>Incremental pull via Search since last_pull_cursor</t>
+          <t>Incremental pull via cursor since last_pull_cursor</t>
         </is>
       </c>
       <c r="D18" s="24" t="inlineStr">
@@ -1750,10 +1754,14 @@
       </c>
       <c r="E18" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F18" s="24" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F18" s="24" t="inlineStr">
+        <is>
+          <t>Verified 2026-07-21 vs mock: incremental pull filters last_edited_time on_or_after last_pull_cursor (per-database query, chosen over Search to scope precisely); no-change pass fetched 0, a remote edit was picked up (updated=1); cursor persists in sync_meta. Clean records take remote; dirty records skipped for Phase 4 reconcile.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="23" t="inlineStr">
@@ -1778,10 +1786,14 @@
       </c>
       <c r="E19" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F19" s="24" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F19" s="24" t="inlineStr">
+        <is>
+          <t>Verified 2026-07-21 vs mock: accounts + income/expense categories upserted from Notion by notion_page_id; selectors and derived balances reflect pulled reference data. sync.now = push+pull; sync.initialPull for onboarding; Sync UI gains initial-pull + push/pull steps.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="23" t="inlineStr">

</xml_diff>

<commit_message>
feat: impl phase 4 desktop app
</commit_message>
<xml_diff>
--- a/wiki/desktop/desktop-development-plan.xlsx
+++ b/wiki/desktop/desktop-development-plan.xlsx
@@ -691,7 +691,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Offline-first Electron desktop client. Local SQLite is the source of truth; Notion is a bidirectional mirror. Phases 0-3 complete on 2026-07-21: usable offline app + full Notion sync — connect (keychain token), schema verify, push, and initial + incremental pull (verified vs a mock Notion API). Milestone M2 (backup sync) done. Next: Phase 4 (three-way merge + conflict resolver).</t>
+          <t>Offline-first Electron desktop client. Local SQLite is the source of truth; Notion is a bidirectional mirror. Phases 0-4 complete on 2026-07-21: usable offline app + FULL bidirectional sync with three-way merge, conflict resolver, sync modes, status badges, and crash/429 durability (verified vs a mock Notion API). Milestone M3 (full sync) done. Only Phase 5 (packaging) remains.</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       </c>
       <c r="D5" s="5">
         <f>COUNTIF('Development Plan'!$E$5:$E$100,"Done")</f>
-        <v>15</v>
+        <v>19</v>
         <v/>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="F5" s="6">
         <f>IFERROR(D5/B5,0)</f>
-        <v>0.681818181818</v>
+        <v>0.863636363636</v>
         <v/>
       </c>
     </row>
@@ -914,7 +914,7 @@
       </c>
       <c r="C13" s="9">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 4",'Development Plan'!$E$5:$E$100,"Not Started")</f>
-        <v>4</v>
+        <v>0</v>
         <v/>
       </c>
       <c r="D13" s="9">
@@ -924,7 +924,7 @@
       </c>
       <c r="E13" s="9">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 4",'Development Plan'!$E$5:$E$100,"Done")</f>
-        <v>0</v>
+        <v>4</v>
         <v/>
       </c>
       <c r="F13" s="9">
@@ -978,7 +978,7 @@
       </c>
       <c r="C15" s="11">
         <f>SUM(C9:C14)</f>
-        <v>7</v>
+        <v>3</v>
         <v/>
       </c>
       <c r="D15" s="11">
@@ -988,7 +988,7 @@
       </c>
       <c r="E15" s="11">
         <f>SUM(E9:E14)</f>
-        <v>15</v>
+        <v>19</v>
         <v/>
       </c>
       <c r="F15" s="11">
@@ -1118,12 +1118,12 @@
       </c>
       <c r="D21" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 4",'Development Plan'!$E$5:$E$100,"Done")</f>
-        <v>0</v>
+        <v>4</v>
         <v/>
       </c>
       <c r="E21" s="15">
         <f>IFERROR(D21/C21,0)</f>
-        <v>0.0</v>
+        <v>1.0</v>
         <v/>
       </c>
       <c r="F21" s="16" t="inlineStr">
@@ -1818,10 +1818,14 @@
       </c>
       <c r="E20" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F20" s="24" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F20" s="24" t="inlineStr">
+        <is>
+          <t>Verified 2026-07-21: pure threeWayMerge (noop/pull/push/automerge/conflict); disjoint fields auto-merge, same-field overlaps conflict; base advances per field. Full scenario-matrix unit tests + live run (conflict base 50k/local 60k/remote 70k; disjoint auto-merge).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="23" t="inlineStr">
@@ -1846,10 +1850,14 @@
       </c>
       <c r="E21" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F21" s="24" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F21" s="24" t="inlineStr">
+        <is>
+          <t>Verified 2026-07-21: reconcile runs pull-before-push (never clobbers remote); overlaps logged to conflicts table + sync_state=conflict; resolver UI (per-field or keep-all-mine/Notion). Live: conflict flagged, resolve keep-local → dirty → pushed → clean, no conflicts left.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="23" t="inlineStr">
@@ -1874,10 +1882,14 @@
       </c>
       <c r="E22" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F22" s="24" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F22" s="24" t="inlineStr">
+        <is>
+          <t>Verified 2026-07-21: manual/auto interval scheduler (net.isOnline gating); SyncStatus adds online/mode/intervalSeconds; global sidebar chip (online, unsynced/conflict counts, last synced, spinner) + per-record dirty/conflict badges per offline-and-state-model.md.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="23" t="inlineStr">
@@ -1902,10 +1914,14 @@
       </c>
       <c r="E23" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F23" s="24" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F23" s="24" t="inlineStr">
+        <is>
+          <t>Verified 2026-07-21: offline edits journaled to mutation_queue and survive as dirty rows (crash-safe via SQLite); push after 'restart' created the record while absorbing an injected 429 via exponential backoff; second push idempotent (0 created).</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="23" t="inlineStr">

</xml_diff>

<commit_message>
feat: impl phase 5
</commit_message>
<xml_diff>
--- a/wiki/desktop/desktop-development-plan.xlsx
+++ b/wiki/desktop/desktop-development-plan.xlsx
@@ -141,7 +141,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -177,11 +177,55 @@
         <color rgb="00E4E7EB"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E4E7EB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E4E7EB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E4E7EB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E4E7EB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E4E7EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E4E7EB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E4E7EB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E4E7EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -251,6 +295,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -691,7 +737,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Offline-first Electron desktop client. Local SQLite is the source of truth; Notion is a bidirectional mirror. Phases 0-4 complete on 2026-07-21: usable offline app + FULL bidirectional sync with three-way merge, conflict resolver, sync modes, status badges, and crash/429 durability (verified vs a mock Notion API). Milestone M3 (full sync) done. Only Phase 5 (packaging) remains.</t>
+          <t>Offline-first Electron desktop client. Local SQLite is the source of truth; Notion is a bidirectional mirror. ALL PHASES COMPLETE (0-5) on 2026-07-21: usable offline app, full bidirectional sync with three-way merge + conflict resolver, and packaged unsigned installers with an Electron e2e suite. Shippable v0.1.0.</t>
         </is>
       </c>
     </row>
@@ -720,7 +766,7 @@
       </c>
       <c r="D5" s="5">
         <f>COUNTIF('Development Plan'!$E$5:$E$100,"Done")</f>
-        <v>19</v>
+        <v>22</v>
         <v/>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -730,7 +776,7 @@
       </c>
       <c r="F5" s="6">
         <f>IFERROR(D5/B5,0)</f>
-        <v>0.863636363636</v>
+        <v>1.0</v>
         <v/>
       </c>
     </row>
@@ -774,192 +820,192 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>Phase 0 — Scaffold &amp; shared logic</t>
         </is>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="14">
         <f>COUNTIF('Development Plan'!$A$5:$A$100,"Phase 0")</f>
         <v>4</v>
         <v/>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 0",'Development Plan'!$E$5:$E$100,"Not Started")</f>
         <v>0</v>
         <v/>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 0",'Development Plan'!$E$5:$E$100,"In Progress")</f>
         <v>0</v>
         <v/>
       </c>
-      <c r="E9" s="9">
+      <c r="E9" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 0",'Development Plan'!$E$5:$E$100,"Done")</f>
         <v>4</v>
         <v/>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 0",'Development Plan'!$E$5:$E$100,"Blocked")</f>
         <v>0</v>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Phase 1 — Offline app (fully usable, no sync)</t>
         </is>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="14">
         <f>COUNTIF('Development Plan'!$A$5:$A$100,"Phase 1")</f>
         <v>5</v>
         <v/>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 1",'Development Plan'!$E$5:$E$100,"Not Started")</f>
         <v>0</v>
         <v/>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 1",'Development Plan'!$E$5:$E$100,"In Progress")</f>
         <v>0</v>
         <v/>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 1",'Development Plan'!$E$5:$E$100,"Done")</f>
         <v>5</v>
         <v/>
       </c>
-      <c r="F10" s="9">
+      <c r="F10" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 1",'Development Plan'!$E$5:$E$100,"Blocked")</f>
         <v>0</v>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>Phase 2 — Onboarding + Push</t>
         </is>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="14">
         <f>COUNTIF('Development Plan'!$A$5:$A$100,"Phase 2")</f>
         <v>3</v>
         <v/>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 2",'Development Plan'!$E$5:$E$100,"Not Started")</f>
         <v>0</v>
         <v/>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 2",'Development Plan'!$E$5:$E$100,"In Progress")</f>
         <v>0</v>
         <v/>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 2",'Development Plan'!$E$5:$E$100,"Done")</f>
         <v>3</v>
         <v/>
       </c>
-      <c r="F11" s="9">
+      <c r="F11" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 2",'Development Plan'!$E$5:$E$100,"Blocked")</f>
         <v>0</v>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>Phase 3 — Pull</t>
         </is>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="14">
         <f>COUNTIF('Development Plan'!$A$5:$A$100,"Phase 3")</f>
         <v>3</v>
         <v/>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 3",'Development Plan'!$E$5:$E$100,"Not Started")</f>
         <v>0</v>
         <v/>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 3",'Development Plan'!$E$5:$E$100,"In Progress")</f>
         <v>0</v>
         <v/>
       </c>
-      <c r="E12" s="9">
+      <c r="E12" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 3",'Development Plan'!$E$5:$E$100,"Done")</f>
         <v>3</v>
         <v/>
       </c>
-      <c r="F12" s="9">
+      <c r="F12" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 3",'Development Plan'!$E$5:$E$100,"Blocked")</f>
         <v>0</v>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>Phase 4 — Reconcile + Conflict</t>
         </is>
       </c>
-      <c r="B13" s="9">
+      <c r="B13" s="14">
         <f>COUNTIF('Development Plan'!$A$5:$A$100,"Phase 4")</f>
         <v>4</v>
         <v/>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 4",'Development Plan'!$E$5:$E$100,"Not Started")</f>
         <v>0</v>
         <v/>
       </c>
-      <c r="D13" s="9">
+      <c r="D13" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 4",'Development Plan'!$E$5:$E$100,"In Progress")</f>
         <v>0</v>
         <v/>
       </c>
-      <c r="E13" s="9">
+      <c r="E13" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 4",'Development Plan'!$E$5:$E$100,"Done")</f>
         <v>4</v>
         <v/>
       </c>
-      <c r="F13" s="9">
+      <c r="F13" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 4",'Development Plan'!$E$5:$E$100,"Blocked")</f>
         <v>0</v>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>Phase 5 — Package</t>
         </is>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="14">
         <f>COUNTIF('Development Plan'!$A$5:$A$100,"Phase 5")</f>
         <v>3</v>
         <v/>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 5",'Development Plan'!$E$5:$E$100,"Not Started")</f>
-        <v>3</v>
-        <v/>
-      </c>
-      <c r="D14" s="9">
+        <v>0</v>
+        <v/>
+      </c>
+      <c r="D14" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 5",'Development Plan'!$E$5:$E$100,"In Progress")</f>
         <v>0</v>
         <v/>
       </c>
-      <c r="E14" s="9">
+      <c r="E14" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 5",'Development Plan'!$E$5:$E$100,"Done")</f>
-        <v>0</v>
-        <v/>
-      </c>
-      <c r="F14" s="9">
+        <v>3</v>
+        <v/>
+      </c>
+      <c r="F14" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 5",'Development Plan'!$E$5:$E$100,"Blocked")</f>
         <v>0</v>
         <v/>
@@ -978,7 +1024,7 @@
       </c>
       <c r="C15" s="11">
         <f>SUM(C9:C14)</f>
-        <v>3</v>
+        <v>0</v>
         <v/>
       </c>
       <c r="D15" s="11">
@@ -988,7 +1034,7 @@
       </c>
       <c r="E15" s="11">
         <f>SUM(E9:E14)</f>
-        <v>19</v>
+        <v>22</v>
         <v/>
       </c>
       <c r="F15" s="11">
@@ -1150,12 +1196,12 @@
       </c>
       <c r="D22" s="14">
         <f>COUNTIFS('Development Plan'!$A$5:$A$100,"Phase 5",'Development Plan'!$E$5:$E$100,"Done")</f>
-        <v>0</v>
+        <v>3</v>
         <v/>
       </c>
       <c r="E22" s="15">
         <f>IFERROR(D22/C22,0)</f>
-        <v>0.0</v>
+        <v>1.0</v>
         <v/>
       </c>
       <c r="F22" s="16" t="inlineStr">
@@ -1182,10 +1228,10 @@
           <t>Planned but not yet begun.</t>
         </is>
       </c>
-      <c r="C25" s="19" t="n"/>
-      <c r="D25" s="19" t="n"/>
-      <c r="E25" s="19" t="n"/>
-      <c r="F25" s="19" t="n"/>
+      <c r="C25" s="25" t="n"/>
+      <c r="D25" s="25" t="n"/>
+      <c r="E25" s="25" t="n"/>
+      <c r="F25" s="26" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="20" t="inlineStr">
@@ -1198,10 +1244,10 @@
           <t>Actively being worked; acceptance not yet met.</t>
         </is>
       </c>
-      <c r="C26" s="19" t="n"/>
-      <c r="D26" s="19" t="n"/>
-      <c r="E26" s="19" t="n"/>
-      <c r="F26" s="19" t="n"/>
+      <c r="C26" s="25" t="n"/>
+      <c r="D26" s="25" t="n"/>
+      <c r="E26" s="25" t="n"/>
+      <c r="F26" s="26" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="21" t="inlineStr">
@@ -1214,10 +1260,10 @@
           <t>Complete and verified against its acceptance criterion.</t>
         </is>
       </c>
-      <c r="C27" s="19" t="n"/>
-      <c r="D27" s="19" t="n"/>
-      <c r="E27" s="19" t="n"/>
-      <c r="F27" s="19" t="n"/>
+      <c r="C27" s="25" t="n"/>
+      <c r="D27" s="25" t="n"/>
+      <c r="E27" s="25" t="n"/>
+      <c r="F27" s="26" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="22" t="inlineStr">
@@ -1230,10 +1276,10 @@
           <t>Cannot proceed without a dependency, decision, or access.</t>
         </is>
       </c>
-      <c r="C28" s="19" t="n"/>
-      <c r="D28" s="19" t="n"/>
-      <c r="E28" s="19" t="n"/>
-      <c r="F28" s="19" t="n"/>
+      <c r="C28" s="25" t="n"/>
+      <c r="D28" s="25" t="n"/>
+      <c r="E28" s="25" t="n"/>
+      <c r="F28" s="26" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -1946,10 +1992,14 @@
       </c>
       <c r="E24" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F24" s="24" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F24" s="24" t="inlineStr">
+        <is>
+          <t>Verified 2026-07-21: electron-builder.yml (mac dmg/zip, linux AppImage, win NSIS), migrations bundled as extraResources, native *.node asarUnpack. Produced arm64 .dmg + .zip (127M); better-sqlite3 rebuilt for packaged Electron ABI; unsigned .app boots (db ready, 11 tables). Win/Linux build on their own platforms/CI.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="23" t="inlineStr">
@@ -1974,10 +2024,14 @@
       </c>
       <c r="E25" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F25" s="24" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F25" s="24" t="inlineStr">
+        <is>
+          <t>Verified 2026-07-21: Playwright _electron drives the built app in isolated userData (seeded reference data). 5/5 green: boot + 9 sections, offline sync chip, seeded accounts with balances, offline income create -&gt; dirty badge -&gt; live dashboard update, multi-window.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="23" t="inlineStr">
@@ -2002,10 +2056,14 @@
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F26" s="24" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F26" s="24" t="inlineStr">
+        <is>
+          <t>notable-finance-app/CHANGELOG.md documents Phases 0-5 at v0.1.0 (Keep a Changelog / SemVer); package.json version 0.1.0. Git tag v0.1.0 deferred to the commit/release step (command noted for the owner).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>